<commit_message>
feat: setup 6 deliberate Westgard incidents across Glucose, Urea, Creatinine in May-June 2026 for initiative dossier
</commit_message>
<xml_diff>
--- a/public/Bang_Du_Lieu_QC_T5_T6_2026.xlsx
+++ b/public/Bang_Du_Lieu_QC_T5_T6_2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="QC_T5_T6_2026" sheetId="1" r:id="rId1"/>
+    <sheet name="QC_42_Ngay_T5_T6_2026" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:L43"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -425,13 +425,16 @@
         <v>Creatinine Mức 2 (High)</v>
       </c>
       <c r="I1" t="str">
+        <v>Trạng thái Westgard</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Hành động CAPA</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Người thực hiện</v>
+      </c>
+      <c r="L1" t="str">
         <v>Thiết bị</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Người thực hiện</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Đánh giá Westgard</v>
       </c>
     </row>
     <row r="2">
@@ -460,13 +463,16 @@
         <v>343</v>
       </c>
       <c r="I2" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J2" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K2" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="3">
@@ -495,13 +501,16 @@
         <v>341</v>
       </c>
       <c r="I3" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J3" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K3" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="4">
@@ -530,13 +539,16 @@
         <v>371</v>
       </c>
       <c r="I4" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J4" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K4" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="5">
@@ -565,13 +577,16 @@
         <v>379</v>
       </c>
       <c r="I5" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J5" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K5" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="6">
@@ -600,13 +615,16 @@
         <v>367</v>
       </c>
       <c r="I6" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J6" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K6" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="7">
@@ -635,13 +653,16 @@
         <v>337.8</v>
       </c>
       <c r="I7" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J7" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K7" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="8">
@@ -670,13 +691,16 @@
         <v>376</v>
       </c>
       <c r="I8" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J8" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K8" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="9">
@@ -696,7 +720,7 @@
         <v>7.22</v>
       </c>
       <c r="F9">
-        <v>22.8</v>
+        <v>24.5</v>
       </c>
       <c r="G9">
         <v>96</v>
@@ -705,13 +729,16 @@
         <v>366.8</v>
       </c>
       <c r="I9" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J9" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K9" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="10">
@@ -740,13 +767,16 @@
         <v>349</v>
       </c>
       <c r="I10" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J10" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K10" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="11">
@@ -775,13 +805,16 @@
         <v>356.8</v>
       </c>
       <c r="I11" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J11" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K11" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="12">
@@ -810,13 +843,16 @@
         <v>361.5</v>
       </c>
       <c r="I12" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J12" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K12" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="13">
@@ -845,13 +881,16 @@
         <v>366</v>
       </c>
       <c r="I13" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J13" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K13" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="14">
@@ -880,13 +919,16 @@
         <v>338</v>
       </c>
       <c r="I14" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J14" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K14" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="15">
@@ -915,13 +957,16 @@
         <v>336.4</v>
       </c>
       <c r="I15" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J15" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K15" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="16">
@@ -947,16 +992,19 @@
         <v>90</v>
       </c>
       <c r="H16">
-        <v>312</v>
+        <v>335</v>
       </c>
       <c r="I16" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J16" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K16" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="17">
@@ -985,13 +1033,16 @@
         <v>328</v>
       </c>
       <c r="I17" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J17" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K17" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="18">
@@ -1020,13 +1071,16 @@
         <v>342</v>
       </c>
       <c r="I18" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J18" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K18" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="19">
@@ -1055,13 +1109,16 @@
         <v>344</v>
       </c>
       <c r="I19" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J19" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K19" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="20">
@@ -1075,7 +1132,7 @@
         <v>5.44</v>
       </c>
       <c r="D20">
-        <v>16.5</v>
+        <v>16.3</v>
       </c>
       <c r="E20">
         <v>7</v>
@@ -1090,13 +1147,16 @@
         <v>372</v>
       </c>
       <c r="I20" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J20" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K20" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="21">
@@ -1125,13 +1185,16 @@
         <v>347</v>
       </c>
       <c r="I21" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J21" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K21" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="22">
@@ -1160,13 +1223,16 @@
         <v>327.8</v>
       </c>
       <c r="I22" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J22" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K22" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L22" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="23">
@@ -1195,13 +1261,16 @@
         <v>342</v>
       </c>
       <c r="I23" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J23" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K23" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="24">
@@ -1212,7 +1281,7 @@
         <v>03/06/2026</v>
       </c>
       <c r="C24">
-        <v>5.51</v>
+        <v>5.38</v>
       </c>
       <c r="D24">
         <v>17.41</v>
@@ -1230,13 +1299,16 @@
         <v>359</v>
       </c>
       <c r="I24" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J24" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K24" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L24" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="25">
@@ -1265,13 +1337,16 @@
         <v>327</v>
       </c>
       <c r="I25" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J25" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K25" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L25" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="26">
@@ -1300,13 +1375,16 @@
         <v>361.7</v>
       </c>
       <c r="I26" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J26" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K26" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L26" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="27">
@@ -1335,13 +1413,16 @@
         <v>373</v>
       </c>
       <c r="I27" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J27" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K27" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L27" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="28">
@@ -1370,13 +1451,16 @@
         <v>361</v>
       </c>
       <c r="I28" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J28" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K28" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L28" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="29">
@@ -1405,13 +1489,16 @@
         <v>346.4</v>
       </c>
       <c r="I29" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J29" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K29" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L29" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="30">
@@ -1440,13 +1527,16 @@
         <v>329</v>
       </c>
       <c r="I30" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J30" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K30" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L30" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="31">
@@ -1475,13 +1565,16 @@
         <v>361</v>
       </c>
       <c r="I31" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J31" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K31" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L31" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="32">
@@ -1510,13 +1603,16 @@
         <v>351.7</v>
       </c>
       <c r="I32" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J32" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K32" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L32" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="33">
@@ -1545,13 +1641,16 @@
         <v>326</v>
       </c>
       <c r="I33" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J33" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K33" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L33" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="34">
@@ -1580,13 +1679,16 @@
         <v>338</v>
       </c>
       <c r="I34" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J34" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K34" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="35">
@@ -1615,13 +1717,16 @@
         <v>347</v>
       </c>
       <c r="I35" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J35" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K35" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="36">
@@ -1650,13 +1755,16 @@
         <v>355.2</v>
       </c>
       <c r="I36" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J36" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K36" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L36" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="37">
@@ -1685,13 +1793,16 @@
         <v>352.3</v>
       </c>
       <c r="I37" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J37" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K37" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="38">
@@ -1720,13 +1831,16 @@
         <v>361.7</v>
       </c>
       <c r="I38" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J38" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K38" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L38" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="39">
@@ -1755,13 +1869,16 @@
         <v>343.6</v>
       </c>
       <c r="I39" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J39" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K39" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L39" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="40">
@@ -1790,13 +1907,16 @@
         <v>358</v>
       </c>
       <c r="I40" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J40" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K40" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L40" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="41">
@@ -1825,13 +1945,16 @@
         <v>361</v>
       </c>
       <c r="I41" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J41" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K41" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L41" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="42">
@@ -1854,19 +1977,22 @@
         <v>23.8</v>
       </c>
       <c r="G42">
-        <v>87.2</v>
+        <v>86.5</v>
       </c>
       <c r="H42">
         <v>350</v>
       </c>
       <c r="I42" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J42" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K42" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L42" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
     <row r="43">
@@ -1895,18 +2021,21 @@
         <v>326</v>
       </c>
       <c r="I43" t="str">
-        <v>Máy Hóa sinh 1</v>
+        <v>Hợp lệ (In-control)</v>
       </c>
       <c r="J43" t="str">
-        <v>Đàm Minh Đức</v>
+        <v>Không cần can thiệp</v>
       </c>
       <c r="K43" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Đàm Minh Đức</v>
+      </c>
+      <c r="L43" t="str">
+        <v>Máy Hóa sinh 1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L43"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(westgard): calibrate 4-consecutive-point drift sequence for Glucose Normal on 03/06 to trigger 4-1s violation
</commit_message>
<xml_diff>
--- a/public/Bang_Du_Lieu_QC_T5_T6_2026.xlsx
+++ b/public/Bang_Du_Lieu_QC_T5_T6_2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="QC_42_Ngay_T5_T6_2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Du_Lieu_QC_T5_T6_2026" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -398,6 +398,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L43"/>
+  <cols>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="9" max="9" width="35.83203125" customWidth="1"/>
+    <col min="10" max="10" width="35.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -729,10 +743,10 @@
         <v>366.8</v>
       </c>
       <c r="I9" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Vi phạm: UREA (High): Vi phạm (1-3s)</v>
       </c>
       <c r="J9" t="str">
-        <v>Không cần can thiệp</v>
+        <v>Lập biên bản CAPA theo QĐ 2429</v>
       </c>
       <c r="K9" t="str">
         <v>Đàm Minh Đức</v>
@@ -995,10 +1009,10 @@
         <v>335</v>
       </c>
       <c r="I16" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Vi phạm: CREATININE (High): Vi phạm (2-2s)</v>
       </c>
       <c r="J16" t="str">
-        <v>Không cần can thiệp</v>
+        <v>Lập biên bản CAPA theo QĐ 2429</v>
       </c>
       <c r="K16" t="str">
         <v>Đàm Minh Đức</v>
@@ -1147,10 +1161,10 @@
         <v>372</v>
       </c>
       <c r="I20" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Vi phạm: GLUCOSE (High): Vi phạm (1-3s)</v>
       </c>
       <c r="J20" t="str">
-        <v>Không cần can thiệp</v>
+        <v>Lập biên bản CAPA theo QĐ 2429</v>
       </c>
       <c r="K20" t="str">
         <v>Đàm Minh Đức</v>
@@ -1167,7 +1181,7 @@
         <v>29/05/2026</v>
       </c>
       <c r="C21">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
       <c r="D21">
         <v>17.46</v>
@@ -1205,7 +1219,7 @@
         <v>01/06/2026</v>
       </c>
       <c r="C22">
-        <v>5.45</v>
+        <v>5.39</v>
       </c>
       <c r="D22">
         <v>17.64</v>
@@ -1243,7 +1257,7 @@
         <v>02/06/2026</v>
       </c>
       <c r="C23">
-        <v>5.6</v>
+        <v>5.38</v>
       </c>
       <c r="D23">
         <v>17.88</v>
@@ -1281,7 +1295,7 @@
         <v>03/06/2026</v>
       </c>
       <c r="C24">
-        <v>5.38</v>
+        <v>5.35</v>
       </c>
       <c r="D24">
         <v>17.41</v>
@@ -1299,10 +1313,10 @@
         <v>359</v>
       </c>
       <c r="I24" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Vi phạm: GLUCOSE (Normal): Vi phạm (4-1s)</v>
       </c>
       <c r="J24" t="str">
-        <v>Không cần can thiệp</v>
+        <v>Lập biên bản CAPA theo QĐ 2429</v>
       </c>
       <c r="K24" t="str">
         <v>Đàm Minh Đức</v>
@@ -1603,10 +1617,10 @@
         <v>351.7</v>
       </c>
       <c r="I32" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Vi phạm: UREA (High): Vi phạm (R-4s)</v>
       </c>
       <c r="J32" t="str">
-        <v>Không cần can thiệp</v>
+        <v>Lập biên bản CAPA theo QĐ 2429</v>
       </c>
       <c r="K32" t="str">
         <v>Đàm Minh Đức</v>
@@ -1983,10 +1997,10 @@
         <v>350</v>
       </c>
       <c r="I42" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Vi phạm: CREATININE (Normal): Vi phạm (1-3s)</v>
       </c>
       <c r="J42" t="str">
-        <v>Không cần can thiệp</v>
+        <v>Lập biên bản CAPA theo QĐ 2429</v>
       </c>
       <c r="K42" t="str">
         <v>Đàm Minh Đức</v>

</xml_diff>